<commit_message>
Make admin catalog edits and bulk import reflect live on the storefront.
Sync PDP gallery on product updates, default bulk import to update-by-SKU, bust homepage and Redis catalog caches on writes, and serve category bento from Postgres. Adds admin rate-limit tuning, zip image import, and E2E coverage for product edit persistence.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/templates/vibemusic-bulk.xlsx
+++ b/docs/templates/vibemusic-bulk.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BQ1"/>
+  <dimension ref="A1:CC1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -607,10 +607,46 @@
       <c r="BQ1" t="str">
         <v>Item Weight Unit</v>
       </c>
+      <c r="BR1" t="str">
+        <v>image1</v>
+      </c>
+      <c r="BS1" t="str">
+        <v>image2</v>
+      </c>
+      <c r="BT1" t="str">
+        <v>image3</v>
+      </c>
+      <c r="BU1" t="str">
+        <v>image4</v>
+      </c>
+      <c r="BV1" t="str">
+        <v>image5</v>
+      </c>
+      <c r="BW1" t="str">
+        <v>image6</v>
+      </c>
+      <c r="BX1" t="str">
+        <v>image7</v>
+      </c>
+      <c r="BY1" t="str">
+        <v>image8</v>
+      </c>
+      <c r="BZ1" t="str">
+        <v>image9</v>
+      </c>
+      <c r="CA1" t="str">
+        <v>image10</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>image11</v>
+      </c>
+      <c r="CC1" t="str">
+        <v>image12</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BQ1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:CC1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>